<commit_message>
(docs): initial user manual + team self assessment and task assignment readme
</commit_message>
<xml_diff>
--- a/docs/sprint2/PI-2024-25_Team-Self-Assessment_v05.xlsx
+++ b/docs/sprint2/PI-2024-25_Team-Self-Assessment_v05.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\IdeaProjects\lapr2\docs\sprint2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD549D54-E054-490C-8369-5792F6A80A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51B6D49-9AFA-430C-9DB8-8B7C69C65E43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Group and Self Assessment" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="59">
   <si>
     <t>TeamID #</t>
   </si>
@@ -212,6 +212,24 @@
   </si>
   <si>
     <t>US12</t>
+  </si>
+  <si>
+    <t>US13</t>
+  </si>
+  <si>
+    <t>US14</t>
+  </si>
+  <si>
+    <t>US15</t>
+  </si>
+  <si>
+    <t>US16</t>
+  </si>
+  <si>
+    <t>US17</t>
+  </si>
+  <si>
+    <t>US18</t>
   </si>
 </sst>
 </file>
@@ -2463,7 +2481,9 @@
       </c>
     </row>
     <row r="18" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="11"/>
+      <c r="A18" s="11" t="s">
+        <v>53</v>
+      </c>
       <c r="B18" s="18"/>
       <c r="C18" s="18"/>
       <c r="D18" s="40"/>
@@ -2487,7 +2507,9 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="11"/>
+      <c r="A19" s="11" t="s">
+        <v>54</v>
+      </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
       <c r="D19" s="40"/>
@@ -2511,9 +2533,15 @@
       </c>
     </row>
     <row r="20" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="11"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
+      <c r="A20" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="18">
+        <v>1241176</v>
+      </c>
+      <c r="C20" s="18">
+        <v>5</v>
+      </c>
       <c r="D20" s="40"/>
       <c r="E20" s="11" t="s">
         <v>27</v>
@@ -2535,9 +2563,15 @@
       </c>
     </row>
     <row r="21" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="11"/>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
+      <c r="A21" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="18">
+        <v>1241323</v>
+      </c>
+      <c r="C21" s="18">
+        <v>5</v>
+      </c>
       <c r="D21" s="40"/>
       <c r="E21" s="11" t="s">
         <v>27</v>
@@ -2559,9 +2593,15 @@
       </c>
     </row>
     <row r="22" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="11"/>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
+      <c r="A22" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="18">
+        <v>1241285</v>
+      </c>
+      <c r="C22" s="18">
+        <v>5</v>
+      </c>
       <c r="D22" s="40"/>
       <c r="E22" s="11" t="s">
         <v>27</v>
@@ -2583,9 +2623,15 @@
       </c>
     </row>
     <row r="23" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="11"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
+      <c r="A23" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" s="18">
+        <v>1241166</v>
+      </c>
+      <c r="C23" s="18">
+        <v>5</v>
+      </c>
       <c r="D23" s="40"/>
       <c r="E23" s="11" t="s">
         <v>27</v>
@@ -2607,9 +2653,15 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A24" s="11"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
+      <c r="A24" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="18">
+        <v>1220804</v>
+      </c>
+      <c r="C24" s="18">
+        <v>5</v>
+      </c>
       <c r="D24" s="40"/>
       <c r="E24" s="11" t="s">
         <v>27</v>
@@ -2751,9 +2803,7 @@
       </c>
     </row>
     <row r="30" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A30" s="11" t="s">
-        <v>40</v>
-      </c>
+      <c r="A30" s="11"/>
       <c r="B30" s="18"/>
       <c r="C30" s="18"/>
       <c r="D30" s="40"/>
@@ -2858,21 +2908,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005836243B3C47804EAF5FFDD9F066FCC7" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d21ddf3f0b128e39c9d770c8c903166">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0326308c339679ad994635f2c691325" ns2:_="">
     <xsd:import namespace="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
@@ -3056,31 +3091,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B77F7C-EE47-4FBD-B078-6536C1487A1E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3096,4 +3122,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
(docs): finished user manual + team self assessment
</commit_message>
<xml_diff>
--- a/docs/sprint2/PI-2024-25_Team-Self-Assessment_v05.xlsx
+++ b/docs/sprint2/PI-2024-25_Team-Self-Assessment_v05.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\IdeaProjects\lapr2\docs\sprint2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51B6D49-9AFA-430C-9DB8-8B7C69C65E43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FB3E96-C9FB-4BD1-A8A6-997F8E596D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Group and Self Assessment" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="60">
   <si>
     <t>TeamID #</t>
   </si>
@@ -230,6 +230,9 @@
   </si>
   <si>
     <t>US18</t>
+  </si>
+  <si>
+    <t>Student 1241176 also developed this US</t>
   </si>
 </sst>
 </file>
@@ -2484,9 +2487,15 @@
       <c r="A18" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="40"/>
+      <c r="B18" s="18">
+        <v>1241166</v>
+      </c>
+      <c r="C18" s="18">
+        <v>5</v>
+      </c>
+      <c r="D18" s="40" t="s">
+        <v>59</v>
+      </c>
       <c r="E18" s="11" t="s">
         <v>27</v>
       </c>
@@ -2510,8 +2519,12 @@
       <c r="A19" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
+      <c r="B19" s="18">
+        <v>1241323</v>
+      </c>
+      <c r="C19" s="18">
+        <v>5</v>
+      </c>
       <c r="D19" s="40"/>
       <c r="E19" s="11" t="s">
         <v>27</v>
@@ -2908,6 +2921,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005836243B3C47804EAF5FFDD9F066FCC7" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d21ddf3f0b128e39c9d770c8c903166">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0326308c339679ad994635f2c691325" ns2:_="">
     <xsd:import namespace="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
@@ -3091,22 +3119,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B77F7C-EE47-4FBD-B078-6536C1487A1E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3122,28 +3159,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>